<commit_message>
chore(data-release): publish site data 2026-09-18 03:51:01 UTC
</commit_message>
<xml_diff>
--- a/countries/bg/2020-2025.xlsx
+++ b/countries/bg/2020-2025.xlsx
@@ -83654,17 +83654,17 @@
       </c>
       <c r="H424" t="inlineStr">
         <is>
-          <t>D017</t>
+          <t>D007</t>
         </is>
       </c>
       <c r="I424" t="inlineStr">
         <is>
-          <t>Measles</t>
+          <t>Hepatitis A</t>
         </is>
       </c>
       <c r="J424" t="inlineStr">
         <is>
-          <t>麻疹</t>
+          <t>甲型肝炎</t>
         </is>
       </c>
       <c r="K424" t="inlineStr">
@@ -83683,13 +83683,13 @@
         </is>
       </c>
       <c r="N424" t="n">
-        <v>2</v>
+        <v>102</v>
       </c>
       <c r="O424" t="n">
-        <v>2</v>
+        <v>102</v>
       </c>
       <c r="R424" t="n">
-        <v>0.02978601947007841</v>
+        <v>1.519086992973999</v>
       </c>
       <c r="S424" t="inlineStr">
         <is>
@@ -83698,7 +83698,7 @@
       </c>
       <c r="U424" t="inlineStr">
         <is>
-          <t>SER_BG_ECDC_MEAS_ANNUAL</t>
+          <t>SER_BG_ECDC_HEPA_ANNUAL</t>
         </is>
       </c>
       <c r="AA424" t="inlineStr">
@@ -83723,7 +83723,7 @@
       </c>
       <c r="AS424" t="inlineStr">
         <is>
-          <t>SER_BG_ECDC_MEAS_ANNUAL</t>
+          <t>SER_BG_ECDC_HEPA_ANNUAL</t>
         </is>
       </c>
       <c r="AT424" t="n">
@@ -83813,17 +83813,17 @@
       </c>
       <c r="H425" t="inlineStr">
         <is>
-          <t>D017</t>
+          <t>D007</t>
         </is>
       </c>
       <c r="I425" t="inlineStr">
         <is>
-          <t>Measles</t>
+          <t>Hepatitis A</t>
         </is>
       </c>
       <c r="J425" t="inlineStr">
         <is>
-          <t>麻疹</t>
+          <t>甲型肝炎</t>
         </is>
       </c>
       <c r="K425" t="inlineStr">
@@ -83842,19 +83842,19 @@
         </is>
       </c>
       <c r="N425" t="n">
-        <v>2</v>
+        <v>102</v>
       </c>
       <c r="O425" t="n">
-        <v>2</v>
+        <v>102</v>
       </c>
       <c r="U425" t="inlineStr">
         <is>
-          <t>SER_BG_ECDC_MEAS_ANNUAL</t>
+          <t>SER_BG_ECDC_HEPA_ANNUAL</t>
         </is>
       </c>
       <c r="V425" t="inlineStr">
         <is>
-          <t>SER_BG_ECDC_MEAS_ANNUAL</t>
+          <t>SER_BG_ECDC_HEPA_ANNUAL</t>
         </is>
       </c>
       <c r="W425" t="inlineStr">
@@ -83864,7 +83864,7 @@
       </c>
       <c r="X425" t="inlineStr">
         <is>
-          <t>Measles</t>
+          <t>Hepatitis A</t>
         </is>
       </c>
       <c r="Y425" t="inlineStr">
@@ -83957,7 +83957,7 @@
       </c>
       <c r="AS425" t="inlineStr">
         <is>
-          <t>SER_BG_ECDC_MEAS_ANNUAL</t>
+          <t>SER_BG_ECDC_HEPA_ANNUAL</t>
         </is>
       </c>
       <c r="AT425" t="n">
@@ -84047,17 +84047,17 @@
       </c>
       <c r="H426" t="inlineStr">
         <is>
-          <t>D040</t>
+          <t>D017</t>
         </is>
       </c>
       <c r="I426" t="inlineStr">
         <is>
-          <t>Rubella</t>
+          <t>Measles</t>
         </is>
       </c>
       <c r="J426" t="inlineStr">
         <is>
-          <t>风疹</t>
+          <t>麻疹</t>
         </is>
       </c>
       <c r="K426" t="inlineStr">
@@ -84076,13 +84076,13 @@
         </is>
       </c>
       <c r="N426" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O426" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R426" t="n">
-        <v>0</v>
+        <v>0.02978601947007841</v>
       </c>
       <c r="S426" t="inlineStr">
         <is>
@@ -84091,7 +84091,7 @@
       </c>
       <c r="U426" t="inlineStr">
         <is>
-          <t>SER_BG_ECDC_RUBE_ANNUAL</t>
+          <t>SER_BG_ECDC_MEAS_ANNUAL</t>
         </is>
       </c>
       <c r="AA426" t="inlineStr">
@@ -84116,7 +84116,7 @@
       </c>
       <c r="AS426" t="inlineStr">
         <is>
-          <t>SER_BG_ECDC_RUBE_ANNUAL</t>
+          <t>SER_BG_ECDC_MEAS_ANNUAL</t>
         </is>
       </c>
       <c r="AT426" t="n">
@@ -84206,17 +84206,17 @@
       </c>
       <c r="H427" t="inlineStr">
         <is>
-          <t>D040</t>
+          <t>D017</t>
         </is>
       </c>
       <c r="I427" t="inlineStr">
         <is>
-          <t>Rubella</t>
+          <t>Measles</t>
         </is>
       </c>
       <c r="J427" t="inlineStr">
         <is>
-          <t>风疹</t>
+          <t>麻疹</t>
         </is>
       </c>
       <c r="K427" t="inlineStr">
@@ -84235,19 +84235,19 @@
         </is>
       </c>
       <c r="N427" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O427" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U427" t="inlineStr">
         <is>
-          <t>SER_BG_ECDC_RUBE_ANNUAL</t>
+          <t>SER_BG_ECDC_MEAS_ANNUAL</t>
         </is>
       </c>
       <c r="V427" t="inlineStr">
         <is>
-          <t>SER_BG_ECDC_RUBE_ANNUAL</t>
+          <t>SER_BG_ECDC_MEAS_ANNUAL</t>
         </is>
       </c>
       <c r="W427" t="inlineStr">
@@ -84257,7 +84257,7 @@
       </c>
       <c r="X427" t="inlineStr">
         <is>
-          <t>Rubella</t>
+          <t>Measles</t>
         </is>
       </c>
       <c r="Y427" t="inlineStr">
@@ -84350,7 +84350,7 @@
       </c>
       <c r="AS427" t="inlineStr">
         <is>
-          <t>SER_BG_ECDC_RUBE_ANNUAL</t>
+          <t>SER_BG_ECDC_MEAS_ANNUAL</t>
         </is>
       </c>
       <c r="AT427" t="n">
@@ -84440,17 +84440,17 @@
       </c>
       <c r="H428" t="inlineStr">
         <is>
-          <t>D107</t>
+          <t>D032</t>
         </is>
       </c>
       <c r="I428" t="inlineStr">
         <is>
-          <t>Legionellosis</t>
+          <t>Brucellosis</t>
         </is>
       </c>
       <c r="J428" t="inlineStr">
         <is>
-          <t>军团菌病</t>
+          <t>布鲁氏菌病</t>
         </is>
       </c>
       <c r="K428" t="inlineStr">
@@ -84469,13 +84469,13 @@
         </is>
       </c>
       <c r="N428" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="O428" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="R428" t="n">
-        <v>0.3276462141708626</v>
+        <v>0.08935805841023525</v>
       </c>
       <c r="S428" t="inlineStr">
         <is>
@@ -84484,7 +84484,7 @@
       </c>
       <c r="U428" t="inlineStr">
         <is>
-          <t>SER_BG_ECDC_LEGI_ANNUAL</t>
+          <t>SER_BG_ECDC_BRUC_ANNUAL</t>
         </is>
       </c>
       <c r="AA428" t="inlineStr">
@@ -84509,7 +84509,7 @@
       </c>
       <c r="AS428" t="inlineStr">
         <is>
-          <t>SER_BG_ECDC_LEGI_ANNUAL</t>
+          <t>SER_BG_ECDC_BRUC_ANNUAL</t>
         </is>
       </c>
       <c r="AT428" t="n">
@@ -84599,17 +84599,17 @@
       </c>
       <c r="H429" t="inlineStr">
         <is>
-          <t>D107</t>
+          <t>D032</t>
         </is>
       </c>
       <c r="I429" t="inlineStr">
         <is>
-          <t>Legionellosis</t>
+          <t>Brucellosis</t>
         </is>
       </c>
       <c r="J429" t="inlineStr">
         <is>
-          <t>军团菌病</t>
+          <t>布鲁氏菌病</t>
         </is>
       </c>
       <c r="K429" t="inlineStr">
@@ -84628,19 +84628,19 @@
         </is>
       </c>
       <c r="N429" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="O429" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="U429" t="inlineStr">
         <is>
-          <t>SER_BG_ECDC_LEGI_ANNUAL</t>
+          <t>SER_BG_ECDC_BRUC_ANNUAL</t>
         </is>
       </c>
       <c r="V429" t="inlineStr">
         <is>
-          <t>SER_BG_ECDC_LEGI_ANNUAL</t>
+          <t>SER_BG_ECDC_BRUC_ANNUAL</t>
         </is>
       </c>
       <c r="W429" t="inlineStr">
@@ -84650,7 +84650,7 @@
       </c>
       <c r="X429" t="inlineStr">
         <is>
-          <t>Legionnaires' disease</t>
+          <t>Brucellosis</t>
         </is>
       </c>
       <c r="Y429" t="inlineStr">
@@ -84743,7 +84743,7 @@
       </c>
       <c r="AS429" t="inlineStr">
         <is>
-          <t>SER_BG_ECDC_LEGI_ANNUAL</t>
+          <t>SER_BG_ECDC_BRUC_ANNUAL</t>
         </is>
       </c>
       <c r="AT429" t="n">
@@ -84790,6 +84790,3936 @@
         </is>
       </c>
       <c r="BC429" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t>D040</t>
+        </is>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>Rubella</t>
+        </is>
+      </c>
+      <c r="J430" t="inlineStr">
+        <is>
+          <t>风疹</t>
+        </is>
+      </c>
+      <c r="K430" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L430" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M430" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N430" t="n">
+        <v>0</v>
+      </c>
+      <c r="O430" t="n">
+        <v>0</v>
+      </c>
+      <c r="R430" t="n">
+        <v>0</v>
+      </c>
+      <c r="S430" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U430" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_RUBE_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA430" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO430" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP430" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ430" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS430" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_RUBE_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT430" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU430" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV430" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="AW430" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="AX430" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="AY430" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+      <c r="AZ430" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="BA430" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="BB430" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="BC430" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t>D040</t>
+        </is>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>Rubella</t>
+        </is>
+      </c>
+      <c r="J431" t="inlineStr">
+        <is>
+          <t>风疹</t>
+        </is>
+      </c>
+      <c r="K431" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L431" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M431" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N431" t="n">
+        <v>0</v>
+      </c>
+      <c r="O431" t="n">
+        <v>0</v>
+      </c>
+      <c r="U431" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_RUBE_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V431" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_RUBE_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W431" t="inlineStr">
+        <is>
+          <t>SRC_BG_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X431" t="inlineStr">
+        <is>
+          <t>Rubella</t>
+        </is>
+      </c>
+      <c r="Y431" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z431" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA431" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB431" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC431" t="inlineStr">
+        <is>
+          <t>country:BG:national</t>
+        </is>
+      </c>
+      <c r="AD431" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE431" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF431" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG431" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH431" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI431" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ431" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK431" t="inlineStr">
+        <is>
+          <t>Bulgaria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM431" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN431" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO431" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP431" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ431" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS431" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_RUBE_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT431" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU431" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV431" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="AW431" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="AX431" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="AY431" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+      <c r="AZ431" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="BA431" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="BB431" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="BC431" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t>D045</t>
+        </is>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>Echinococcosis</t>
+        </is>
+      </c>
+      <c r="J432" t="inlineStr">
+        <is>
+          <t>包虫病</t>
+        </is>
+      </c>
+      <c r="K432" t="inlineStr">
+        <is>
+          <t>Parasitic</t>
+        </is>
+      </c>
+      <c r="L432" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M432" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N432" t="n">
+        <v>107</v>
+      </c>
+      <c r="O432" t="n">
+        <v>107</v>
+      </c>
+      <c r="R432" t="n">
+        <v>1.593552041649195</v>
+      </c>
+      <c r="S432" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U432" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_ECHI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA432" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO432" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP432" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ432" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS432" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_ECHI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT432" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU432" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV432" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="AW432" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="AX432" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="AY432" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+      <c r="AZ432" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="BA432" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="BB432" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="BC432" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t>D045</t>
+        </is>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>Echinococcosis</t>
+        </is>
+      </c>
+      <c r="J433" t="inlineStr">
+        <is>
+          <t>包虫病</t>
+        </is>
+      </c>
+      <c r="K433" t="inlineStr">
+        <is>
+          <t>Parasitic</t>
+        </is>
+      </c>
+      <c r="L433" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M433" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N433" t="n">
+        <v>107</v>
+      </c>
+      <c r="O433" t="n">
+        <v>107</v>
+      </c>
+      <c r="U433" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_ECHI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V433" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_ECHI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W433" t="inlineStr">
+        <is>
+          <t>SRC_BG_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X433" t="inlineStr">
+        <is>
+          <t>Echinococcosis</t>
+        </is>
+      </c>
+      <c r="Y433" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z433" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA433" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB433" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC433" t="inlineStr">
+        <is>
+          <t>country:BG:national</t>
+        </is>
+      </c>
+      <c r="AD433" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE433" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF433" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG433" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH433" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI433" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ433" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK433" t="inlineStr">
+        <is>
+          <t>Bulgaria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM433" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN433" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO433" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP433" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ433" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS433" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_ECHI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT433" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU433" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV433" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="AW433" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="AX433" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="AY433" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+      <c r="AZ433" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="BA433" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="BB433" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="BC433" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="G434" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="H434" t="inlineStr">
+        <is>
+          <t>D085</t>
+        </is>
+      </c>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>Toxoplasmosis</t>
+        </is>
+      </c>
+      <c r="J434" t="inlineStr">
+        <is>
+          <t>弓形体病</t>
+        </is>
+      </c>
+      <c r="K434" t="inlineStr">
+        <is>
+          <t>Parasitic</t>
+        </is>
+      </c>
+      <c r="L434" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M434" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N434" t="n">
+        <v>0</v>
+      </c>
+      <c r="O434" t="n">
+        <v>0</v>
+      </c>
+      <c r="R434" t="n">
+        <v>0</v>
+      </c>
+      <c r="S434" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U434" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_TOXO_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA434" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO434" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP434" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ434" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS434" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_TOXO_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT434" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU434" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV434" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="AW434" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="AX434" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="AY434" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+      <c r="AZ434" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="BA434" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="BB434" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="BC434" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="G435" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="H435" t="inlineStr">
+        <is>
+          <t>D085</t>
+        </is>
+      </c>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>Toxoplasmosis</t>
+        </is>
+      </c>
+      <c r="J435" t="inlineStr">
+        <is>
+          <t>弓形体病</t>
+        </is>
+      </c>
+      <c r="K435" t="inlineStr">
+        <is>
+          <t>Parasitic</t>
+        </is>
+      </c>
+      <c r="L435" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M435" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N435" t="n">
+        <v>0</v>
+      </c>
+      <c r="O435" t="n">
+        <v>0</v>
+      </c>
+      <c r="U435" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_TOXO_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V435" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_TOXO_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W435" t="inlineStr">
+        <is>
+          <t>SRC_BG_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X435" t="inlineStr">
+        <is>
+          <t>Toxoplasmosis, congenital</t>
+        </is>
+      </c>
+      <c r="Y435" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z435" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA435" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB435" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC435" t="inlineStr">
+        <is>
+          <t>country:BG:national</t>
+        </is>
+      </c>
+      <c r="AD435" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE435" t="inlineStr">
+        <is>
+          <t>narrower</t>
+        </is>
+      </c>
+      <c r="AF435" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG435" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH435" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI435" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ435" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK435" t="inlineStr">
+        <is>
+          <t>Bulgaria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM435" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN435" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO435" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP435" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ435" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS435" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_TOXO_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT435" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU435" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV435" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="AW435" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="AX435" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="AY435" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+      <c r="AZ435" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="BA435" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="BB435" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="BC435" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="G436" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="H436" t="inlineStr">
+        <is>
+          <t>D092</t>
+        </is>
+      </c>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>Campylobacteriosis</t>
+        </is>
+      </c>
+      <c r="J436" t="inlineStr">
+        <is>
+          <t>弯曲杆菌病</t>
+        </is>
+      </c>
+      <c r="K436" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L436" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M436" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N436" t="n">
+        <v>520</v>
+      </c>
+      <c r="O436" t="n">
+        <v>520</v>
+      </c>
+      <c r="R436" t="n">
+        <v>7.744365062220388</v>
+      </c>
+      <c r="S436" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U436" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_CAMP_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA436" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO436" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP436" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ436" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS436" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_CAMP_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT436" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU436" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV436" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="AW436" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="AX436" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="AY436" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+      <c r="AZ436" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="BA436" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="BB436" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="BC436" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>D092</t>
+        </is>
+      </c>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>Campylobacteriosis</t>
+        </is>
+      </c>
+      <c r="J437" t="inlineStr">
+        <is>
+          <t>弯曲杆菌病</t>
+        </is>
+      </c>
+      <c r="K437" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L437" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M437" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N437" t="n">
+        <v>520</v>
+      </c>
+      <c r="O437" t="n">
+        <v>520</v>
+      </c>
+      <c r="U437" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_CAMP_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V437" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_CAMP_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W437" t="inlineStr">
+        <is>
+          <t>SRC_BG_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X437" t="inlineStr">
+        <is>
+          <t>Campylobacteriosis</t>
+        </is>
+      </c>
+      <c r="Y437" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z437" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA437" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB437" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC437" t="inlineStr">
+        <is>
+          <t>country:BG:national</t>
+        </is>
+      </c>
+      <c r="AD437" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE437" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF437" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG437" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH437" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI437" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ437" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK437" t="inlineStr">
+        <is>
+          <t>Bulgaria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM437" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN437" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO437" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP437" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ437" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS437" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_CAMP_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT437" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU437" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV437" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="AW437" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="AX437" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="AY437" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+      <c r="AZ437" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="BA437" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="BB437" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="BC437" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="G438" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="H438" t="inlineStr">
+        <is>
+          <t>D105</t>
+        </is>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>Shigellosis</t>
+        </is>
+      </c>
+      <c r="J438" t="inlineStr">
+        <is>
+          <t>志贺菌病</t>
+        </is>
+      </c>
+      <c r="K438" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L438" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M438" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N438" t="n">
+        <v>61</v>
+      </c>
+      <c r="O438" t="n">
+        <v>61</v>
+      </c>
+      <c r="R438" t="n">
+        <v>0.9084735938373918</v>
+      </c>
+      <c r="S438" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U438" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_SHIG_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA438" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO438" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP438" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ438" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS438" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_SHIG_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT438" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU438" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV438" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="AW438" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="AX438" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="AY438" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+      <c r="AZ438" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="BA438" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="BB438" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="BC438" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="G439" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="H439" t="inlineStr">
+        <is>
+          <t>D105</t>
+        </is>
+      </c>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>Shigellosis</t>
+        </is>
+      </c>
+      <c r="J439" t="inlineStr">
+        <is>
+          <t>志贺菌病</t>
+        </is>
+      </c>
+      <c r="K439" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L439" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M439" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N439" t="n">
+        <v>61</v>
+      </c>
+      <c r="O439" t="n">
+        <v>61</v>
+      </c>
+      <c r="U439" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_SHIG_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V439" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_SHIG_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W439" t="inlineStr">
+        <is>
+          <t>SRC_BG_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X439" t="inlineStr">
+        <is>
+          <t>Shigellosis</t>
+        </is>
+      </c>
+      <c r="Y439" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z439" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA439" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB439" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC439" t="inlineStr">
+        <is>
+          <t>country:BG:national</t>
+        </is>
+      </c>
+      <c r="AD439" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE439" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF439" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG439" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH439" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI439" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ439" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK439" t="inlineStr">
+        <is>
+          <t>Bulgaria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM439" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN439" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO439" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP439" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ439" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS439" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_SHIG_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT439" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU439" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV439" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="AW439" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="AX439" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="AY439" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+      <c r="AZ439" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="BA439" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="BB439" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="BC439" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="G440" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="H440" t="inlineStr">
+        <is>
+          <t>D107</t>
+        </is>
+      </c>
+      <c r="I440" t="inlineStr">
+        <is>
+          <t>Legionellosis</t>
+        </is>
+      </c>
+      <c r="J440" t="inlineStr">
+        <is>
+          <t>军团菌病</t>
+        </is>
+      </c>
+      <c r="K440" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L440" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M440" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N440" t="n">
+        <v>22</v>
+      </c>
+      <c r="O440" t="n">
+        <v>22</v>
+      </c>
+      <c r="R440" t="n">
+        <v>0.3276462141708626</v>
+      </c>
+      <c r="S440" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U440" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_LEGI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA440" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO440" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP440" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ440" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS440" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_LEGI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT440" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU440" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV440" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="AW440" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="AX440" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="AY440" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+      <c r="AZ440" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="BA440" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="BB440" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="BC440" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="G441" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="H441" t="inlineStr">
+        <is>
+          <t>D107</t>
+        </is>
+      </c>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t>Legionellosis</t>
+        </is>
+      </c>
+      <c r="J441" t="inlineStr">
+        <is>
+          <t>军团菌病</t>
+        </is>
+      </c>
+      <c r="K441" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L441" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M441" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N441" t="n">
+        <v>22</v>
+      </c>
+      <c r="O441" t="n">
+        <v>22</v>
+      </c>
+      <c r="U441" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_LEGI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V441" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_LEGI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W441" t="inlineStr">
+        <is>
+          <t>SRC_BG_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X441" t="inlineStr">
+        <is>
+          <t>Legionnaires' disease</t>
+        </is>
+      </c>
+      <c r="Y441" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z441" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA441" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB441" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC441" t="inlineStr">
+        <is>
+          <t>country:BG:national</t>
+        </is>
+      </c>
+      <c r="AD441" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE441" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF441" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG441" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH441" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI441" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ441" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK441" t="inlineStr">
+        <is>
+          <t>Bulgaria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM441" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN441" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO441" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP441" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ441" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS441" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_LEGI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT441" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU441" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV441" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="AW441" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="AX441" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="AY441" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+      <c r="AZ441" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="BA441" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="BB441" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="BC441" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="H442" t="inlineStr">
+        <is>
+          <t>D108</t>
+        </is>
+      </c>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t>Listeriosis</t>
+        </is>
+      </c>
+      <c r="J442" t="inlineStr">
+        <is>
+          <t>李斯特菌病</t>
+        </is>
+      </c>
+      <c r="K442" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L442" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M442" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N442" t="n">
+        <v>6</v>
+      </c>
+      <c r="O442" t="n">
+        <v>6</v>
+      </c>
+      <c r="R442" t="n">
+        <v>0.08935805841023525</v>
+      </c>
+      <c r="S442" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U442" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_LIST_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA442" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO442" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP442" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ442" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS442" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_LIST_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT442" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU442" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV442" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="AW442" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="AX442" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="AY442" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+      <c r="AZ442" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="BA442" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="BB442" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="BC442" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="G443" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="H443" t="inlineStr">
+        <is>
+          <t>D108</t>
+        </is>
+      </c>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t>Listeriosis</t>
+        </is>
+      </c>
+      <c r="J443" t="inlineStr">
+        <is>
+          <t>李斯特菌病</t>
+        </is>
+      </c>
+      <c r="K443" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L443" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M443" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N443" t="n">
+        <v>6</v>
+      </c>
+      <c r="O443" t="n">
+        <v>6</v>
+      </c>
+      <c r="U443" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_LIST_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V443" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_LIST_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W443" t="inlineStr">
+        <is>
+          <t>SRC_BG_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X443" t="inlineStr">
+        <is>
+          <t>Listeriosis</t>
+        </is>
+      </c>
+      <c r="Y443" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z443" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA443" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB443" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC443" t="inlineStr">
+        <is>
+          <t>country:BG:national</t>
+        </is>
+      </c>
+      <c r="AD443" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE443" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF443" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG443" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH443" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI443" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ443" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK443" t="inlineStr">
+        <is>
+          <t>Bulgaria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM443" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN443" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO443" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP443" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ443" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS443" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_LIST_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT443" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU443" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV443" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="AW443" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="AX443" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="AY443" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+      <c r="AZ443" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="BA443" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="BB443" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="BC443" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="G444" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="H444" t="inlineStr">
+        <is>
+          <t>D114</t>
+        </is>
+      </c>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t>Salmonellosis</t>
+        </is>
+      </c>
+      <c r="J444" t="inlineStr">
+        <is>
+          <t>沙门氏菌病</t>
+        </is>
+      </c>
+      <c r="K444" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L444" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M444" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N444" t="n">
+        <v>770</v>
+      </c>
+      <c r="O444" t="n">
+        <v>770</v>
+      </c>
+      <c r="R444" t="n">
+        <v>11.46761749598019</v>
+      </c>
+      <c r="S444" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U444" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_SALM_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA444" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO444" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP444" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ444" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS444" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_SALM_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT444" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU444" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV444" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="AW444" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="AX444" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="AY444" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+      <c r="AZ444" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="BA444" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="BB444" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="BC444" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="G445" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="H445" t="inlineStr">
+        <is>
+          <t>D114</t>
+        </is>
+      </c>
+      <c r="I445" t="inlineStr">
+        <is>
+          <t>Salmonellosis</t>
+        </is>
+      </c>
+      <c r="J445" t="inlineStr">
+        <is>
+          <t>沙门氏菌病</t>
+        </is>
+      </c>
+      <c r="K445" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L445" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M445" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N445" t="n">
+        <v>770</v>
+      </c>
+      <c r="O445" t="n">
+        <v>770</v>
+      </c>
+      <c r="U445" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_SALM_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V445" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_SALM_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W445" t="inlineStr">
+        <is>
+          <t>SRC_BG_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X445" t="inlineStr">
+        <is>
+          <t>Salmonellosis</t>
+        </is>
+      </c>
+      <c r="Y445" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z445" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA445" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB445" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC445" t="inlineStr">
+        <is>
+          <t>country:BG:national</t>
+        </is>
+      </c>
+      <c r="AD445" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE445" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF445" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG445" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH445" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI445" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ445" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK445" t="inlineStr">
+        <is>
+          <t>Bulgaria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM445" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN445" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO445" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP445" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ445" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS445" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_SALM_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT445" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU445" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV445" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="AW445" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="AX445" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="AY445" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+      <c r="AZ445" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="BA445" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="BB445" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="BC445" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="G446" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="H446" t="inlineStr">
+        <is>
+          <t>D115</t>
+        </is>
+      </c>
+      <c r="I446" t="inlineStr">
+        <is>
+          <t>Shiga toxin-producing Escherichia coli infection</t>
+        </is>
+      </c>
+      <c r="J446" t="inlineStr">
+        <is>
+          <t>产志贺毒素大肠杆菌感染</t>
+        </is>
+      </c>
+      <c r="K446" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L446" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M446" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N446" t="n">
+        <v>2</v>
+      </c>
+      <c r="O446" t="n">
+        <v>2</v>
+      </c>
+      <c r="R446" t="n">
+        <v>0.02978601947007841</v>
+      </c>
+      <c r="S446" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U446" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_STEC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA446" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO446" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP446" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ446" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS446" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_STEC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT446" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU446" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV446" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="AW446" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="AX446" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="AY446" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+      <c r="AZ446" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="BA446" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="BB446" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="BC446" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="G447" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="H447" t="inlineStr">
+        <is>
+          <t>D115</t>
+        </is>
+      </c>
+      <c r="I447" t="inlineStr">
+        <is>
+          <t>Shiga toxin-producing Escherichia coli infection</t>
+        </is>
+      </c>
+      <c r="J447" t="inlineStr">
+        <is>
+          <t>产志贺毒素大肠杆菌感染</t>
+        </is>
+      </c>
+      <c r="K447" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L447" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M447" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N447" t="n">
+        <v>2</v>
+      </c>
+      <c r="O447" t="n">
+        <v>2</v>
+      </c>
+      <c r="U447" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_STEC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V447" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_STEC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W447" t="inlineStr">
+        <is>
+          <t>SRC_BG_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X447" t="inlineStr">
+        <is>
+          <t>STEC/VTEC infection</t>
+        </is>
+      </c>
+      <c r="Y447" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z447" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA447" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB447" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC447" t="inlineStr">
+        <is>
+          <t>country:BG:national</t>
+        </is>
+      </c>
+      <c r="AD447" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE447" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF447" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG447" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH447" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI447" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ447" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK447" t="inlineStr">
+        <is>
+          <t>Bulgaria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM447" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN447" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO447" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP447" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ447" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS447" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_STEC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT447" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU447" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV447" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="AW447" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="AX447" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="AY447" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+      <c r="AZ447" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="BA447" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="BB447" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="BC447" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="G448" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="H448" t="inlineStr">
+        <is>
+          <t>D122</t>
+        </is>
+      </c>
+      <c r="I448" t="inlineStr">
+        <is>
+          <t>Trichinellosis</t>
+        </is>
+      </c>
+      <c r="J448" t="inlineStr">
+        <is>
+          <t>旋毛虫病</t>
+        </is>
+      </c>
+      <c r="K448" t="inlineStr">
+        <is>
+          <t>Parasitic</t>
+        </is>
+      </c>
+      <c r="L448" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M448" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N448" t="n">
+        <v>12</v>
+      </c>
+      <c r="O448" t="n">
+        <v>12</v>
+      </c>
+      <c r="R448" t="n">
+        <v>0.1787161168204705</v>
+      </c>
+      <c r="S448" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U448" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_TRIC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA448" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO448" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP448" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ448" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS448" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_TRIC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT448" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU448" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV448" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="AW448" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="AX448" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="AY448" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+      <c r="AZ448" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="BA448" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="BB448" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="BC448" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>bg</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="G449" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="H449" t="inlineStr">
+        <is>
+          <t>D122</t>
+        </is>
+      </c>
+      <c r="I449" t="inlineStr">
+        <is>
+          <t>Trichinellosis</t>
+        </is>
+      </c>
+      <c r="J449" t="inlineStr">
+        <is>
+          <t>旋毛虫病</t>
+        </is>
+      </c>
+      <c r="K449" t="inlineStr">
+        <is>
+          <t>Parasitic</t>
+        </is>
+      </c>
+      <c r="L449" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M449" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N449" t="n">
+        <v>12</v>
+      </c>
+      <c r="O449" t="n">
+        <v>12</v>
+      </c>
+      <c r="U449" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_TRIC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V449" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_TRIC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W449" t="inlineStr">
+        <is>
+          <t>SRC_BG_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X449" t="inlineStr">
+        <is>
+          <t>Trichinellosis</t>
+        </is>
+      </c>
+      <c r="Y449" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z449" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA449" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB449" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC449" t="inlineStr">
+        <is>
+          <t>country:BG:national</t>
+        </is>
+      </c>
+      <c r="AD449" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE449" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF449" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG449" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH449" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI449" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ449" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK449" t="inlineStr">
+        <is>
+          <t>Bulgaria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM449" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN449" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO449" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP449" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ449" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS449" t="inlineStr">
+        <is>
+          <t>SER_BG_ECDC_TRIC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT449" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU449" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV449" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="AW449" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="AX449" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="AY449" t="inlineStr">
+        <is>
+          <t>official_ecdc_rest_aggregate</t>
+        </is>
+      </c>
+      <c r="AZ449" t="inlineStr">
+        <is>
+          <t>ecdc_atlas_annual</t>
+        </is>
+      </c>
+      <c r="BA449" t="inlineStr">
+        <is>
+          <t>ECDC Surveillance Atlas — Bulgaria Annual Baseline</t>
+        </is>
+      </c>
+      <c r="BB449" t="inlineStr">
+        <is>
+          <t>https://atlas.ecdc.europa.eu/public/index.aspx/</t>
+        </is>
+      </c>
+      <c r="BC449" t="inlineStr">
         <is>
           <t>official_ecdc_rest_aggregate</t>
         </is>
@@ -84911,7 +88841,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>214</v>
+        <v>224</v>
       </c>
     </row>
     <row r="10">
@@ -84921,7 +88851,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>428</v>
+        <v>448</v>
       </c>
     </row>
     <row r="11">
@@ -84941,7 +88871,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>214</v>
+        <v>224</v>
       </c>
     </row>
     <row r="13">
@@ -84973,7 +88903,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>19139</v>
+        <v>20725</v>
       </c>
     </row>
     <row r="16">

</xml_diff>